<commit_message>
feat: optimize delivery note generation
</commit_message>
<xml_diff>
--- a/MEDIT_Delivery Note_template.xlsx
+++ b/MEDIT_Delivery Note_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Jueun_workspace\label-parsing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7EDBF90-6978-42A0-8D3C-31C7F32A0D9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE30D45A-82B2-4831-B3A6-FD091E811CB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24780" yWindow="750" windowWidth="24000" windowHeight="14925" xr2:uid="{24D67D64-FC68-4323-89FF-3AA92157D581}"/>
+    <workbookView xWindow="-25680" yWindow="1380" windowWidth="24000" windowHeight="14925" xr2:uid="{24D67D64-FC68-4323-89FF-3AA92157D581}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="59">
   <si>
     <t>ACI_form_202502-04DN</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -289,24 +289,6 @@
   </si>
   <si>
     <t>3A0111853C0</t>
-  </si>
-  <si>
-    <t>Tip check</t>
-  </si>
-  <si>
-    <t>Sum</t>
-  </si>
-  <si>
-    <t>box</t>
-  </si>
-  <si>
-    <t>carton</t>
-  </si>
-  <si>
-    <t>total</t>
-  </si>
-  <si>
-    <t>price</t>
   </si>
   <si>
     <t>Pallets :  1 stk</t>
@@ -431,18 +413,12 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="6">
@@ -521,7 +497,7 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyFill="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -576,12 +552,6 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1113,7 +1083,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{582CACAF-87EC-44FD-AA1A-A45AFFC8D3D9}">
-  <dimension ref="A1:L182"/>
+  <dimension ref="A1:E182"/>
   <sheetFormatPr defaultColWidth="9.33203125" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="30.6640625" style="1" customWidth="1"/>
@@ -1122,14 +1092,10 @@
     <col min="4" max="4" width="35.33203125" style="1" customWidth="1"/>
     <col min="5" max="5" width="31.33203125" style="1" customWidth="1"/>
     <col min="6" max="6" width="10.1640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="9.1640625" style="3" customWidth="1"/>
-    <col min="8" max="8" width="7.5" style="3" customWidth="1"/>
-    <col min="9" max="11" width="9.33203125" style="3"/>
-    <col min="12" max="12" width="11" style="3" customWidth="1"/>
-    <col min="13" max="16384" width="9.33203125" style="1"/>
+    <col min="7" max="16384" width="9.33203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="17.25" customHeight="1">
+    <row r="1" spans="1:5" ht="17.25" customHeight="1">
       <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
@@ -1137,7 +1103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="17.25" customHeight="1">
+    <row r="2" spans="1:5" ht="17.25" customHeight="1">
       <c r="D2" s="12" t="s">
         <v>15</v>
       </c>
@@ -1145,7 +1111,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="17.25" customHeight="1">
+    <row r="3" spans="1:5" ht="17.25" customHeight="1">
       <c r="D3" s="2" t="s">
         <v>3</v>
       </c>
@@ -1153,17 +1119,17 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="17.25" customHeight="1">
-      <c r="A4" s="24" t="e" vm="1">
+    <row r="4" spans="1:5" ht="17.25" customHeight="1">
+      <c r="A4" s="22" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="24"/>
-    </row>
-    <row r="5" spans="1:12" ht="36.75" customHeight="1">
-      <c r="A5" s="24"/>
-      <c r="B5" s="24"/>
-      <c r="C5" s="24"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+    </row>
+    <row r="5" spans="1:5" ht="36.75" customHeight="1">
+      <c r="A5" s="22"/>
+      <c r="B5" s="22"/>
+      <c r="C5" s="22"/>
       <c r="D5" s="4" t="s">
         <v>14</v>
       </c>
@@ -1171,10 +1137,10 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="13.5">
-      <c r="A6" s="24"/>
-      <c r="B6" s="24"/>
-      <c r="C6" s="24"/>
+    <row r="6" spans="1:5" ht="13.5">
+      <c r="A6" s="22"/>
+      <c r="B6" s="22"/>
+      <c r="C6" s="22"/>
       <c r="D6" s="5" t="s">
         <v>5</v>
       </c>
@@ -1182,50 +1148,50 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="17.25" customHeight="1">
-      <c r="A7" s="24"/>
-      <c r="B7" s="24"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="21"/>
-      <c r="E7" s="22"/>
-    </row>
-    <row r="8" spans="1:12" ht="17.25" customHeight="1">
-      <c r="A8" s="24"/>
-      <c r="B8" s="24"/>
-      <c r="C8" s="24"/>
-      <c r="D8" s="22"/>
-      <c r="E8" s="22"/>
-    </row>
-    <row r="9" spans="1:12" ht="28.5" customHeight="1">
-      <c r="A9" s="24"/>
-      <c r="B9" s="24"/>
-      <c r="C9" s="24"/>
-      <c r="D9" s="23"/>
-      <c r="E9" s="23"/>
-    </row>
-    <row r="10" spans="1:12">
+    <row r="7" spans="1:5" ht="17.25" customHeight="1">
+      <c r="A7" s="22"/>
+      <c r="B7" s="22"/>
+      <c r="C7" s="22"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="20"/>
+    </row>
+    <row r="8" spans="1:5" ht="17.25" customHeight="1">
+      <c r="A8" s="22"/>
+      <c r="B8" s="22"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="20"/>
+    </row>
+    <row r="9" spans="1:5" ht="28.5" customHeight="1">
+      <c r="A9" s="22"/>
+      <c r="B9" s="22"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="21"/>
+      <c r="E9" s="21"/>
+    </row>
+    <row r="10" spans="1:5">
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
     </row>
-    <row r="11" spans="1:12" s="7" customFormat="1" ht="19.5">
-      <c r="A11" s="9" t="str">
-        <f xml:space="preserve"> "CARTON : " &amp; J14 &amp; " stk"</f>
-        <v>CARTON : 31 stk</v>
-      </c>
-      <c r="B11" s="25" t="s">
-        <v>62</v>
-      </c>
-      <c r="C11" s="25"/>
+    <row r="11" spans="1:5" s="7" customFormat="1" ht="19.5">
+      <c r="A11" s="9" t="e">
+        <f xml:space="preserve"> "CARTON : " &amp;#REF! &amp; " stk"</f>
+        <v>#REF!</v>
+      </c>
+      <c r="B11" s="23" t="s">
+        <v>56</v>
+      </c>
+      <c r="C11" s="23"/>
       <c r="D11" s="9"/>
     </row>
-    <row r="12" spans="1:12">
+    <row r="12" spans="1:5">
       <c r="A12" s="8">
         <f ca="1">TODAY()</f>
-        <v>46185</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" ht="15.75" customHeight="1">
+        <v>46190</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="15.75" customHeight="1">
       <c r="A13" s="13" t="s">
         <v>6</v>
       </c>
@@ -1233,167 +1199,55 @@
         <v>7</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="E13" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="G13" s="19" t="s">
-        <v>56</v>
-      </c>
-      <c r="H13" s="19" t="s">
-        <v>57</v>
-      </c>
-      <c r="I13" s="19" t="s">
-        <v>58</v>
-      </c>
-      <c r="J13" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="K13" s="19" t="s">
-        <v>60</v>
-      </c>
-      <c r="L13" s="19" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="12" customHeight="1">
+    </row>
+    <row r="14" spans="1:5" ht="12" customHeight="1">
       <c r="A14" s="16"/>
       <c r="B14" s="16"/>
       <c r="C14" s="16"/>
       <c r="D14" s="16"/>
       <c r="E14" s="16"/>
-      <c r="G14" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C14)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H14" s="19">
-        <f>SUM(G:G)</f>
-        <v>0</v>
-      </c>
-      <c r="I14" s="19">
-        <v>8</v>
-      </c>
-      <c r="J14" s="20">
-        <v>31</v>
-      </c>
-      <c r="K14" s="19">
-        <f>H14+I14+J14</f>
-        <v>39</v>
-      </c>
-      <c r="L14" s="19">
-        <f>K14 * 0.8</f>
-        <v>31.200000000000003</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12">
-      <c r="G15" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C15)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12">
-      <c r="G16" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C16)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7">
-      <c r="G17" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C17)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="11.25" customHeight="1">
-      <c r="G18" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C18)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="11.25" customHeight="1">
-      <c r="G19" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C19)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="11.25" customHeight="1">
-      <c r="G20" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C20)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7">
-      <c r="G21" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C21)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="11.25" customHeight="1">
+    </row>
+    <row r="18" spans="1:5" ht="11.25" customHeight="1"/>
+    <row r="19" spans="1:5" ht="11.25" customHeight="1"/>
+    <row r="20" spans="1:5" ht="11.25" customHeight="1"/>
+    <row r="22" spans="1:5" ht="11.25" customHeight="1">
       <c r="A22" s="10" t="s">
         <v>11</v>
       </c>
       <c r="D22" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G22" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C22)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="11.25" customHeight="1">
-      <c r="G23" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C23)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="11.25" customHeight="1">
+    </row>
+    <row r="23" spans="1:5" ht="11.25" customHeight="1"/>
+    <row r="24" spans="1:5" ht="11.25" customHeight="1">
       <c r="A24" s="10" t="s">
         <v>9</v>
       </c>
       <c r="D24" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="G24" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C24)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="11.25" customHeight="1">
+    </row>
+    <row r="25" spans="1:5" ht="11.25" customHeight="1">
       <c r="A25" s="10"/>
       <c r="D25" s="10"/>
-      <c r="G25" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C25)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="15.75">
+    </row>
+    <row r="26" spans="1:5" ht="15.75">
       <c r="A26" s="10" t="s">
         <v>10</v>
       </c>
       <c r="D26" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G26" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C26)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7">
-      <c r="G27" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C27)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7">
-      <c r="G28" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C28)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="15.75">
+    </row>
+    <row r="29" spans="1:5" ht="15.75">
       <c r="A29" s="10" t="s">
         <v>12</v>
       </c>
@@ -1403,929 +1257,66 @@
         <v>12</v>
       </c>
       <c r="E29" s="11"/>
-      <c r="G29" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C29)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7">
-      <c r="G30" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C30)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7">
-      <c r="G31" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C31)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7">
-      <c r="G32" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C32)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G33" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C33)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G34" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C34)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G35" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C35)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G36" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C36)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G37" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C37)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G38" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C38)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G39" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C39)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="7:7">
-      <c r="G40" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C40)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="7:7">
-      <c r="G41" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C41)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G42" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C42)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G43" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C43)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G44" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C44)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G45" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C45)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="7:7">
-      <c r="G46" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C46)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="7:7">
-      <c r="G47" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C47)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" spans="7:7">
-      <c r="G48" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C48)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="7:7">
-      <c r="G49" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C49)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="7:7">
-      <c r="G50" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C50)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="7:7">
-      <c r="G51" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C51)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G52" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C52)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="7:7">
-      <c r="G53" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C53)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G54" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C54)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="7:7">
-      <c r="G55" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C55)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G56" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C56)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G57" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C57)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G58" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C58)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G59" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C59)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G60" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C60)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G61" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C61)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G62" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C62)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G63" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C63)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64" spans="7:7">
-      <c r="G64" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C64)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" spans="7:7">
-      <c r="G65" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C65)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66" spans="7:7">
-      <c r="G66" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C66)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67" spans="7:7">
-      <c r="G67" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C67)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68" spans="7:7">
-      <c r="G68" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C68)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69" spans="7:7">
-      <c r="G69" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C69)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70" spans="7:7">
-      <c r="G70" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C70)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G71" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C71)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G72" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C72)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G73" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C73)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G74" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C74)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G75" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C75)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="76" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G76" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C76)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="77" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G77" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C77)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="78" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G78" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C78)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="79" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G79" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C79)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="80" spans="7:7">
-      <c r="G80" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C80)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="81" spans="7:7">
-      <c r="G81" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C81)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="82" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G82" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C82)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="83" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G83" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C83)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="84" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G84" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C84)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="85" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G85" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C85)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="86" spans="7:7">
-      <c r="G86" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C86)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="87" spans="7:7">
-      <c r="G87" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C87)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="88" spans="7:7">
-      <c r="G88" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C88)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="89" spans="7:7">
-      <c r="G89" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C89)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="90" spans="7:7">
-      <c r="G90" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C90)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="91" spans="7:7">
-      <c r="G91" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C91)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="92" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G92" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C92)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="93" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G93" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C93)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="94" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G94" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C94)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="95" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G95" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C95)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="96" spans="7:7">
-      <c r="G96" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C96)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="97" spans="7:7">
-      <c r="G97" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C97)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="98" spans="7:7">
-      <c r="G98" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C98)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="99" spans="7:7">
-      <c r="G99" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C99)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="100" spans="7:7">
-      <c r="G100" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C100)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="101" spans="7:7">
-      <c r="G101" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C101)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="102" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G102" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C102)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="103" spans="7:7">
-      <c r="G103" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C103)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="104" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G104" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C104)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="105" spans="7:7">
-      <c r="G105" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C105)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="106" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G106" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C106)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="107" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G107" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C107)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="108" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G108" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C108)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="109" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G109" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C109)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="110" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G110" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C110)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="111" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G111" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C111)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="112" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G112" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C112)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="113" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G113" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C113)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="114" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G114" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C114)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="115" spans="7:7" ht="11.25" customHeight="1">
-      <c r="G115" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C115)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="116" spans="7:7">
-      <c r="G116" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C116)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="117" spans="7:7">
-      <c r="G117" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C117)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="118" spans="7:7">
-      <c r="G118" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C118)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="119" spans="7:7">
-      <c r="G119" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C119)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="120" spans="7:7">
-      <c r="G120" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C120)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="121" spans="7:7">
-      <c r="G121" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C121)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="122" spans="7:7">
-      <c r="G122" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C122)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="123" spans="7:7">
-      <c r="G123" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C123)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="124" spans="7:7">
-      <c r="G124" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C124)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="125" spans="7:7">
-      <c r="G125" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C125)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="126" spans="7:7">
-      <c r="G126" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C126)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="127" spans="7:7">
-      <c r="G127" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C127)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="128" spans="7:7">
-      <c r="G128" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C128)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="129" spans="7:7">
-      <c r="G129" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C129)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="130" spans="7:7">
-      <c r="G130" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C130)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="131" spans="7:7">
-      <c r="G131" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C131)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="132" spans="7:7">
-      <c r="G132" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C132)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="133" spans="7:7">
-      <c r="G133" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C133)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="134" spans="7:7">
-      <c r="G134" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C134)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="135" spans="7:7">
-      <c r="G135" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C135)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="136" spans="7:7">
-      <c r="G136" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C136)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="137" spans="7:7">
-      <c r="G137" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C137)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="138" spans="7:7">
-      <c r="G138" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C138)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="139" spans="7:7">
-      <c r="G139" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C139)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="140" spans="7:7">
-      <c r="G140" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C140)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="141" spans="7:7">
-      <c r="G141" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C141)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="142" spans="7:7">
-      <c r="G142" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C142)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="143" spans="7:7">
-      <c r="G143" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C143)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="144" spans="7:7">
-      <c r="G144" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C144)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="145" spans="7:7">
-      <c r="G145" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C145)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="146" spans="7:7">
-      <c r="G146" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C146)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="147" spans="7:7">
-      <c r="G147" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C147)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="148" spans="7:7">
-      <c r="G148" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C148)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="149" spans="7:7">
-      <c r="G149" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C149)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="150" spans="7:7">
-      <c r="G150" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C150)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="151" spans="7:7">
-      <c r="G151" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C151)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="152" spans="7:7">
-      <c r="G152" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C152)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="153" spans="7:7">
-      <c r="G153" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C153)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="154" spans="7:7">
-      <c r="G154" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C154)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="155" spans="7:7">
-      <c r="G155" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C155)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="156" spans="7:7">
-      <c r="G156" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C156)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="157" spans="7:7">
-      <c r="G157" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C157)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="158" spans="7:7">
-      <c r="G158" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C158)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="159" spans="7:7">
-      <c r="G159" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C159)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="160" spans="7:7">
-      <c r="G160" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C160)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="161" spans="7:7">
-      <c r="G161" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C161)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="162" spans="7:7">
-      <c r="G162" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C162)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="163" spans="7:7">
-      <c r="G163" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C163)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="164" spans="7:7" ht="12" customHeight="1">
-      <c r="G164" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C164)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="165" spans="7:7">
-      <c r="G165" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C165)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="166" spans="7:7">
-      <c r="G166" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C166)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="167" spans="7:7">
-      <c r="G167" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C167)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="168" spans="7:7">
-      <c r="G168" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C168)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="169" spans="7:7">
-      <c r="G169" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C169)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="170" spans="7:7">
-      <c r="G170" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C170)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="171" spans="7:7">
-      <c r="G171" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C171)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="172" spans="7:7">
-      <c r="G172" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C172)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="173" spans="7:7">
-      <c r="G173" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C173)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="174" spans="7:7">
-      <c r="G174" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C174)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="175" spans="7:7" ht="15" customHeight="1">
-      <c r="G175" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C175)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="176" spans="7:7" ht="15" customHeight="1">
-      <c r="G176" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C176)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="177" spans="7:7" ht="15" customHeight="1">
-      <c r="G177" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C177)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="178" spans="7:7" ht="15" customHeight="1">
-      <c r="G178" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C178)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="179" spans="7:7" ht="15" customHeight="1">
-      <c r="G179" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C179)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="180" spans="7:7" ht="15" customHeight="1">
-      <c r="G180" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C180)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="181" spans="7:7" ht="15" customHeight="1">
-      <c r="G181" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C181)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="182" spans="7:7" ht="15" customHeight="1">
-      <c r="G182" s="3">
-        <f>IF(COUNTIF(Sheet2!C:C,C182)&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="33" ht="11.25" customHeight="1"/>
+    <row r="34" ht="11.25" customHeight="1"/>
+    <row r="35" ht="11.25" customHeight="1"/>
+    <row r="36" ht="11.25" customHeight="1"/>
+    <row r="37" ht="11.25" customHeight="1"/>
+    <row r="38" ht="11.25" customHeight="1"/>
+    <row r="39" ht="11.25" customHeight="1"/>
+    <row r="42" ht="11.25" customHeight="1"/>
+    <row r="43" ht="11.25" customHeight="1"/>
+    <row r="44" ht="11.25" customHeight="1"/>
+    <row r="45" ht="11.25" customHeight="1"/>
+    <row r="52" ht="11.25" customHeight="1"/>
+    <row r="54" ht="11.25" customHeight="1"/>
+    <row r="56" ht="11.25" customHeight="1"/>
+    <row r="57" ht="11.25" customHeight="1"/>
+    <row r="58" ht="11.25" customHeight="1"/>
+    <row r="59" ht="11.25" customHeight="1"/>
+    <row r="60" ht="11.25" customHeight="1"/>
+    <row r="61" ht="11.25" customHeight="1"/>
+    <row r="62" ht="11.25" customHeight="1"/>
+    <row r="63" ht="11.25" customHeight="1"/>
+    <row r="71" ht="11.25" customHeight="1"/>
+    <row r="72" ht="11.25" customHeight="1"/>
+    <row r="73" ht="11.25" customHeight="1"/>
+    <row r="74" ht="11.25" customHeight="1"/>
+    <row r="75" ht="11.25" customHeight="1"/>
+    <row r="76" ht="11.25" customHeight="1"/>
+    <row r="77" ht="11.25" customHeight="1"/>
+    <row r="78" ht="11.25" customHeight="1"/>
+    <row r="79" ht="11.25" customHeight="1"/>
+    <row r="82" ht="11.25" customHeight="1"/>
+    <row r="83" ht="11.25" customHeight="1"/>
+    <row r="84" ht="11.25" customHeight="1"/>
+    <row r="85" ht="11.25" customHeight="1"/>
+    <row r="92" ht="11.25" customHeight="1"/>
+    <row r="93" ht="11.25" customHeight="1"/>
+    <row r="94" ht="11.25" customHeight="1"/>
+    <row r="95" ht="11.25" customHeight="1"/>
+    <row r="102" ht="11.25" customHeight="1"/>
+    <row r="104" ht="11.25" customHeight="1"/>
+    <row r="106" ht="11.25" customHeight="1"/>
+    <row r="107" ht="11.25" customHeight="1"/>
+    <row r="108" ht="11.25" customHeight="1"/>
+    <row r="109" ht="11.25" customHeight="1"/>
+    <row r="110" ht="11.25" customHeight="1"/>
+    <row r="111" ht="11.25" customHeight="1"/>
+    <row r="112" ht="11.25" customHeight="1"/>
+    <row r="113" ht="11.25" customHeight="1"/>
+    <row r="114" ht="11.25" customHeight="1"/>
+    <row r="115" ht="11.25" customHeight="1"/>
+    <row r="164" ht="12" customHeight="1"/>
+    <row r="175" ht="15" customHeight="1"/>
+    <row r="176" ht="15" customHeight="1"/>
+    <row r="177" ht="15" customHeight="1"/>
+    <row r="178" ht="15" customHeight="1"/>
+    <row r="179" ht="15" customHeight="1"/>
+    <row r="180" ht="15" customHeight="1"/>
+    <row r="181" ht="15" customHeight="1"/>
+    <row r="182" ht="15" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="D7:D9"/>

</xml_diff>